<commit_message>
feat: implement high-performance Excel import service and support for 50k record processing
</commit_message>
<xml_diff>
--- a/MaintenanceOrders_Template.xlsx
+++ b/MaintenanceOrders_Template.xlsx
@@ -14,10 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="120">
-  <si>
-    <t>Order</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="120">
   <si>
     <t>Equipment</t>
   </si>
@@ -49,9 +46,6 @@
     <t>Materials (Inline Optional)</t>
   </si>
   <si>
-    <t>MO-2001</t>
-  </si>
-  <si>
     <t>EQ-001</t>
   </si>
   <si>
@@ -76,205 +70,211 @@
     <t>2026-09-15</t>
   </si>
   <si>
+    <t>10:Visual pump inspection:2; 20:Dismantle housing:3.5; 30:Reassemble &amp; test:2</t>
+  </si>
+  <si>
+    <t>MAT-001:2; MAT-003:5</t>
+  </si>
+  <si>
+    <t>EQ-002</t>
+  </si>
+  <si>
+    <t>Motor Bearing Check &amp; Alignment</t>
+  </si>
+  <si>
+    <t>2000</t>
+  </si>
+  <si>
+    <t>CORRECTIVE</t>
+  </si>
+  <si>
+    <t>MEDIUM</t>
+  </si>
+  <si>
+    <t>SARAH</t>
+  </si>
+  <si>
+    <t>2026-09-12</t>
+  </si>
+  <si>
+    <t>2026-09-18</t>
+  </si>
+  <si>
+    <t>10:Measure bearing temp:1.5; 20:Grease motor bearings:1</t>
+  </si>
+  <si>
+    <t>MAT-001:1; MAT-003:2</t>
+  </si>
+  <si>
+    <t>EQ-003</t>
+  </si>
+  <si>
+    <t>Emergency Valve Fix &amp; Replacement</t>
+  </si>
+  <si>
+    <t>3000</t>
+  </si>
+  <si>
+    <t>EMERGENCY</t>
+  </si>
+  <si>
+    <t>CRITICAL</t>
+  </si>
+  <si>
+    <t>ALEX</t>
+  </si>
+  <si>
+    <t>2026-09-05</t>
+  </si>
+  <si>
+    <t>10:Isolate valve:1; 20:Replace valve core &amp; seals:4</t>
+  </si>
+  <si>
+    <t>MAT-002:1; MAT-005:8</t>
+  </si>
+  <si>
+    <t>EQ-004</t>
+  </si>
+  <si>
+    <t>Conveyor Belt Tension Tuning</t>
+  </si>
+  <si>
+    <t>LOW</t>
+  </si>
+  <si>
+    <t>2026-09-20</t>
+  </si>
+  <si>
+    <t>2026-09-25</t>
+  </si>
+  <si>
+    <t>10:Tension Check:2; 20:Alignment:1</t>
+  </si>
+  <si>
+    <t>MAT-005:10</t>
+  </si>
+  <si>
+    <t>EQ-005</t>
+  </si>
+  <si>
+    <t>Turbine Lubricant &amp; Filter Service</t>
+  </si>
+  <si>
+    <t>2026-09-22</t>
+  </si>
+  <si>
+    <t>10:Drain Oil:1; 20:Refill Lubricant:2</t>
+  </si>
+  <si>
+    <t>MAT-003:5; MAT-002:1</t>
+  </si>
+  <si>
+    <t>OperationNo</t>
+  </si>
+  <si>
+    <t>WorkCenter</t>
+  </si>
+  <si>
+    <t>Technician</t>
+  </si>
+  <si>
+    <t>PlannedHours</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Visual pump inspection &amp; vibration test</t>
+  </si>
+  <si>
+    <t>WC-001</t>
+  </si>
+  <si>
+    <t>T-001</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>Dismantle housing and check seals</t>
+  </si>
+  <si>
+    <t>WC-002</t>
+  </si>
+  <si>
+    <t>T-002</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>Reassemble and conduct pressure test</t>
+  </si>
+  <si>
+    <t>WC-003</t>
+  </si>
+  <si>
+    <t>T-003</t>
+  </si>
+  <si>
+    <t>Measure motor bearing temperature</t>
+  </si>
+  <si>
+    <t>Grease motor bearings</t>
+  </si>
+  <si>
+    <t>Shut down pipeline &amp; isolate valve</t>
+  </si>
+  <si>
+    <t>Replace broken valve core and seals</t>
+  </si>
+  <si>
+    <t>Material</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>MAT-001</t>
+  </si>
+  <si>
+    <t>EA</t>
+  </si>
+  <si>
+    <t>MAT-003</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>MAT-002</t>
+  </si>
+  <si>
+    <t>MAT-005</t>
+  </si>
+  <si>
+    <t>SET</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Code / Key</t>
+  </si>
+  <si>
+    <t>Description / Details</t>
+  </si>
+  <si>
+    <t>Unit Price (USD)</t>
+  </si>
+  <si>
+    <t>Centrifugal Pump A1 (Plant 1000)</t>
+  </si>
+  <si>
     <t/>
-  </si>
-  <si>
-    <t>MO-2002</t>
-  </si>
-  <si>
-    <t>EQ-002</t>
-  </si>
-  <si>
-    <t>Motor Bearing Check &amp; Alignment</t>
-  </si>
-  <si>
-    <t>2000</t>
-  </si>
-  <si>
-    <t>CORRECTIVE</t>
-  </si>
-  <si>
-    <t>MEDIUM</t>
-  </si>
-  <si>
-    <t>SARAH</t>
-  </si>
-  <si>
-    <t>2026-09-12</t>
-  </si>
-  <si>
-    <t>2026-09-18</t>
-  </si>
-  <si>
-    <t>MO-2003</t>
-  </si>
-  <si>
-    <t>EQ-003</t>
-  </si>
-  <si>
-    <t>Emergency Valve Fix &amp; Replacement</t>
-  </si>
-  <si>
-    <t>3000</t>
-  </si>
-  <si>
-    <t>EMERGENCY</t>
-  </si>
-  <si>
-    <t>CRITICAL</t>
-  </si>
-  <si>
-    <t>ALEX</t>
-  </si>
-  <si>
-    <t>2026-09-05</t>
-  </si>
-  <si>
-    <t>MO-2004</t>
-  </si>
-  <si>
-    <t>EQ-004</t>
-  </si>
-  <si>
-    <t>Conveyor Belt Tension Tuning</t>
-  </si>
-  <si>
-    <t>LOW</t>
-  </si>
-  <si>
-    <t>2026-09-20</t>
-  </si>
-  <si>
-    <t>2026-09-25</t>
-  </si>
-  <si>
-    <t>10:Tension Check:2; 20:Alignment:1</t>
-  </si>
-  <si>
-    <t>MAT-005:10</t>
-  </si>
-  <si>
-    <t>MO-2005</t>
-  </si>
-  <si>
-    <t>EQ-005</t>
-  </si>
-  <si>
-    <t>Turbine Lubricant &amp; Filter Service</t>
-  </si>
-  <si>
-    <t>2026-09-22</t>
-  </si>
-  <si>
-    <t>10:Drain Oil:1; 20:Refill Lubricant:2</t>
-  </si>
-  <si>
-    <t>MAT-003:5; MAT-002:1</t>
-  </si>
-  <si>
-    <t>OperationNo</t>
-  </si>
-  <si>
-    <t>WorkCenter</t>
-  </si>
-  <si>
-    <t>Technician</t>
-  </si>
-  <si>
-    <t>PlannedHours</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>Visual pump inspection &amp; vibration test</t>
-  </si>
-  <si>
-    <t>WC-001</t>
-  </si>
-  <si>
-    <t>T-001</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>Dismantle housing and check seals</t>
-  </si>
-  <si>
-    <t>WC-002</t>
-  </si>
-  <si>
-    <t>T-002</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>Reassemble and conduct pressure test</t>
-  </si>
-  <si>
-    <t>WC-003</t>
-  </si>
-  <si>
-    <t>T-003</t>
-  </si>
-  <si>
-    <t>Measure motor bearing temperature</t>
-  </si>
-  <si>
-    <t>Grease motor bearings</t>
-  </si>
-  <si>
-    <t>Shut down pipeline &amp; isolate valve</t>
-  </si>
-  <si>
-    <t>Replace broken valve core and seals</t>
-  </si>
-  <si>
-    <t>Material</t>
-  </si>
-  <si>
-    <t>Quantity</t>
-  </si>
-  <si>
-    <t>Unit</t>
-  </si>
-  <si>
-    <t>MAT-001</t>
-  </si>
-  <si>
-    <t>EA</t>
-  </si>
-  <si>
-    <t>MAT-003</t>
-  </si>
-  <si>
-    <t>L</t>
-  </si>
-  <si>
-    <t>MAT-002</t>
-  </si>
-  <si>
-    <t>MAT-005</t>
-  </si>
-  <si>
-    <t>SET</t>
-  </si>
-  <si>
-    <t>Category</t>
-  </si>
-  <si>
-    <t>Code / Key</t>
-  </si>
-  <si>
-    <t>Description / Details</t>
-  </si>
-  <si>
-    <t>Unit Price (USD)</t>
-  </si>
-  <si>
-    <t>Centrifugal Pump A1 (Plant 1000)</t>
   </si>
   <si>
     <t>Hydraulic Motor B2 (Plant 2000)</t>
@@ -797,20 +797,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="42" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="9" width="18" customWidth="1"/>
-    <col min="10" max="10" width="36" customWidth="1"/>
-    <col min="11" max="11" width="34" customWidth="1"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="42" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="36" customWidth="1"/>
+    <col min="10" max="10" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="26" customHeight="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -841,88 +841,79 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" ht="20" customHeight="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="2" t="s">
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="K2" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="I3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="J3" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="J3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>32</v>
       </c>
       <c r="D4" s="3" t="s">
@@ -938,86 +929,77 @@
         <v>36</v>
       </c>
       <c r="H4" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I4" s="3" t="s">
-        <v>37</v>
-      </c>
       <c r="J4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="B5" s="2" t="s">
         <v>40</v>
       </c>
+      <c r="C5" s="3" t="s">
+        <v>12</v>
+      </c>
       <c r="D5" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E5" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>41</v>
-      </c>
       <c r="G5" s="3" t="s">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="I5" s="3" t="s">
         <v>43</v>
       </c>
+      <c r="I5" s="2" t="s">
+        <v>44</v>
+      </c>
       <c r="J5" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="K5" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="6" ht="20" customHeight="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" ht="20" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="I6" s="3" t="s">
+      <c r="I6" s="2" t="s">
         <v>49</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1041,36 +1023,36 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>54</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>58</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>59</v>
       </c>
       <c r="F2" s="5">
         <v>2</v>
@@ -1078,19 +1060,19 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>62</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>63</v>
       </c>
       <c r="F3" s="5">
         <v>3.5</v>
@@ -1098,19 +1080,19 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>66</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>67</v>
       </c>
       <c r="F4" s="5">
         <v>2</v>
@@ -1118,19 +1100,19 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D5" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>58</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>59</v>
       </c>
       <c r="F5" s="5">
         <v>1.5</v>
@@ -1138,19 +1120,19 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D6" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>62</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>63</v>
       </c>
       <c r="F6" s="5">
         <v>1</v>
@@ -1161,16 +1143,16 @@
         <v>30</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D7" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E7" s="3" t="s">
         <v>58</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>59</v>
       </c>
       <c r="F7" s="5">
         <v>1</v>
@@ -1181,16 +1163,16 @@
         <v>30</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D8" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>62</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>63</v>
       </c>
       <c r="F8" s="5">
         <v>4</v>
@@ -1218,69 +1200,69 @@
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C1" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="D1" s="6" t="s">
         <v>73</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C2" s="5">
         <v>2</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C3" s="5">
         <v>5</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C4" s="5">
         <v>1</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C5" s="5">
         <v>2</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1288,13 +1270,13 @@
         <v>30</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C6" s="5">
         <v>1</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1302,13 +1284,13 @@
         <v>30</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C7" s="5">
         <v>8</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -1330,63 +1312,63 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="C1" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="D1" s="7" t="s">
         <v>84</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>87</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>88</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>39</v>
@@ -1395,63 +1377,63 @@
         <v>89</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>90</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>91</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>92</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>93</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1459,13 +1441,13 @@
         <v>94</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1473,13 +1455,13 @@
         <v>94</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>96</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1487,18 +1469,18 @@
         <v>94</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>97</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>41</v>
@@ -1507,91 +1489,91 @@
         <v>98</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>99</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>100</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>101</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>102</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>103</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>104</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1599,13 +1581,13 @@
         <v>105</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>106</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1613,13 +1595,13 @@
         <v>105</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>107</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1627,13 +1609,13 @@
         <v>105</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>108</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1641,7 +1623,7 @@
         <v>109</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>110</v>
@@ -1655,7 +1637,7 @@
         <v>109</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>112</v>
@@ -1669,7 +1651,7 @@
         <v>109</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>114</v>
@@ -1697,7 +1679,7 @@
         <v>109</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>118</v>

</xml_diff>